<commit_message>
fix(cloud-estimation): bundle Unicode font for readable PNG labels
</commit_message>
<xml_diff>
--- a/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
+++ b/skill-updates/2026-10-07/cloud-estimation-suite/examples/synthetic-cloud-estimate.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7488CA5D-1A4C-426F-B786-856B7CA0C028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E62B907-BC0A-4C6A-AEB4-5FDC78FF4234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -624,7 +624,7 @@
     <t>JSON</t>
   </si>
   <si>
-    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "e0e2ec9c8c883554d77b86ce2bf5b328b61887fce74c656004457b9ae0aa4bf2", "svg": "24f1d21beb26437d7654dcddffaf415355f953121602a68fd44cdb12ef2c2150"}, "warnings": []}</t>
+    <t>{"edge_ids": ["FLOW-01"], "icon_provenance": [], "icon_sources": ["provider-neutral"], "node_ids": ["COMP-01", "COMP-02", "COMP-03", "COMP-04"], "output_hashes": {"png": "29908a7330c509dfb1b8cf18fb12a5b675699b1297dc0adebe921f692e82afc6", "svg": "71725f3c9a4a48719f40374c8a9b7fbd49ef72762b53d572fab1b6a4e20184eb"}, "warnings": []}</t>
   </si>
   <si>
     <t>Taches_JH</t>

</xml_diff>